<commit_message>
Fix the excel_ALL Bug
</commit_message>
<xml_diff>
--- a/app/dist/main/excel_payment.xlsx
+++ b/app/dist/main/excel_payment.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jackey\Desktop\github\work-order\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3177E884-5B65-41FC-B465-33C7D71D0C12}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0F7C536-1179-4ABB-A312-454F4FC999DF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView showHorizontalScroll="0" showSheetTabs="0" xWindow="32767" yWindow="32767" windowWidth="24180" windowHeight="13053" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,16 +23,13 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="27">
   <si>
     <t>彩意企業有限公司</t>
   </si>
   <si>
     <t>新北市新店區富貴街23巷2號1樓
 TEL:(02)-22145786 FAX:(02)2214-5782</t>
-  </si>
-  <si>
-    <t>報價單</t>
   </si>
   <si>
     <t>客戶名稱:</t>
@@ -111,6 +108,10 @@
   </si>
   <si>
     <t>備料計價</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>報價單</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -118,7 +119,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11">
+  <fonts count="13">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -188,6 +189,17 @@
       <family val="2"/>
       <charset val="136"/>
     </font>
+    <font>
+      <sz val="20"/>
+      <name val="微軟正黑體"/>
+      <family val="2"/>
+      <charset val="136"/>
+    </font>
+    <font>
+      <sz val="20"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -451,7 +463,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -522,21 +534,16 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
@@ -544,11 +551,32 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -559,25 +587,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
@@ -879,137 +901,137 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="33.700000000000003" customHeight="1" thickBot="1">
-      <c r="B1" s="50" t="s">
+      <c r="B1" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
       <c r="E1" s="17"/>
-      <c r="F1" s="51" t="s">
+      <c r="F1" s="41" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-      <c r="K1" s="34" t="s">
-        <v>2</v>
-      </c>
-      <c r="L1" s="29"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
+      <c r="I1" s="40"/>
+      <c r="J1" s="40"/>
+      <c r="K1" s="49" t="s">
+        <v>26</v>
+      </c>
+      <c r="L1" s="40"/>
     </row>
     <row r="2" spans="1:13" ht="17" customHeight="1">
-      <c r="B2" s="48"/>
-      <c r="C2" s="48"/>
-      <c r="D2" s="48"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
       <c r="E2" s="20"/>
-      <c r="F2" s="48"/>
-      <c r="G2" s="48"/>
-      <c r="H2" s="48"/>
-      <c r="I2" s="48"/>
-      <c r="J2" s="48"/>
-      <c r="K2" s="29"/>
-      <c r="L2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="29"/>
+      <c r="J2" s="29"/>
+      <c r="K2" s="40"/>
+      <c r="L2" s="40"/>
     </row>
     <row r="3" spans="1:13" ht="32.700000000000003" customHeight="1">
       <c r="B3" s="21" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="50"/>
+      <c r="D3" s="51"/>
+      <c r="E3" s="52"/>
+      <c r="F3" s="27" t="s">
         <v>3</v>
-      </c>
-      <c r="C3" s="44"/>
-      <c r="D3" s="45"/>
-      <c r="E3" s="46"/>
-      <c r="F3" s="27" t="s">
-        <v>4</v>
       </c>
       <c r="G3" s="24"/>
       <c r="H3" s="21" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I3" s="3"/>
       <c r="J3" s="21" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K3" s="22"/>
       <c r="L3" s="9" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="32.700000000000003" customHeight="1">
       <c r="B4" s="21" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="44"/>
-      <c r="D4" s="45"/>
-      <c r="E4" s="45"/>
-      <c r="F4" s="45"/>
-      <c r="G4" s="46"/>
+        <v>9</v>
+      </c>
+      <c r="C4" s="50"/>
+      <c r="D4" s="51"/>
+      <c r="E4" s="51"/>
+      <c r="F4" s="51"/>
+      <c r="G4" s="52"/>
       <c r="H4" s="23" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I4" s="22"/>
       <c r="J4" s="21" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K4" s="22"/>
-      <c r="L4" s="30"/>
-      <c r="M4" s="28"/>
+      <c r="L4" s="46"/>
+      <c r="M4" s="45"/>
     </row>
     <row r="5" spans="1:13" ht="33" customHeight="1">
       <c r="B5" s="21" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C5" s="22"/>
-      <c r="D5" s="52" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" s="52"/>
-      <c r="F5" s="53"/>
-      <c r="G5" s="53"/>
-      <c r="H5" s="53"/>
-      <c r="I5" s="53"/>
-      <c r="J5" s="53"/>
-      <c r="K5" s="53"/>
-      <c r="L5" s="31"/>
-      <c r="M5" s="29"/>
+      <c r="D5" s="43" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" s="43"/>
+      <c r="F5" s="44"/>
+      <c r="G5" s="44"/>
+      <c r="H5" s="44"/>
+      <c r="I5" s="44"/>
+      <c r="J5" s="44"/>
+      <c r="K5" s="44"/>
+      <c r="L5" s="33"/>
+      <c r="M5" s="40"/>
     </row>
     <row r="6" spans="1:13" ht="30" customHeight="1">
       <c r="A6" s="1"/>
       <c r="B6" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="47" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="32" t="s">
+      <c r="D6" s="48"/>
+      <c r="E6" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="33"/>
-      <c r="E6" s="13" t="s">
+      <c r="F6" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="F6" s="13" t="s">
+      <c r="G6" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="G6" s="14" t="s">
+      <c r="H6" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="H6" s="15" t="s">
+      <c r="I6" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="J6" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="I6" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="J6" s="15" t="s">
+      <c r="K6" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="K6" s="16" t="s">
-        <v>19</v>
-      </c>
       <c r="L6" s="25" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="30" customHeight="1">
       <c r="A7" s="1"/>
       <c r="B7" s="26"/>
-      <c r="C7" s="43"/>
-      <c r="D7" s="43"/>
+      <c r="C7" s="42"/>
+      <c r="D7" s="42"/>
       <c r="E7" s="26"/>
       <c r="F7" s="26"/>
       <c r="G7" s="26"/>
@@ -1022,8 +1044,8 @@
     <row r="8" spans="1:13" ht="30" customHeight="1">
       <c r="A8" s="1"/>
       <c r="B8" s="26"/>
-      <c r="C8" s="43"/>
-      <c r="D8" s="43"/>
+      <c r="C8" s="42"/>
+      <c r="D8" s="42"/>
       <c r="E8" s="26"/>
       <c r="F8" s="26"/>
       <c r="G8" s="26"/>
@@ -1036,8 +1058,8 @@
     <row r="9" spans="1:13" ht="30" customHeight="1">
       <c r="A9" s="1"/>
       <c r="B9" s="26"/>
-      <c r="C9" s="43"/>
-      <c r="D9" s="43"/>
+      <c r="C9" s="42"/>
+      <c r="D9" s="42"/>
       <c r="E9" s="26"/>
       <c r="F9" s="26"/>
       <c r="G9" s="26"/>
@@ -1050,8 +1072,8 @@
     <row r="10" spans="1:13" ht="30" customHeight="1">
       <c r="A10" s="1"/>
       <c r="B10" s="26"/>
-      <c r="C10" s="43"/>
-      <c r="D10" s="43"/>
+      <c r="C10" s="42"/>
+      <c r="D10" s="42"/>
       <c r="E10" s="26"/>
       <c r="F10" s="26"/>
       <c r="G10" s="26"/>
@@ -1064,8 +1086,8 @@
     <row r="11" spans="1:13" ht="30" customHeight="1">
       <c r="A11" s="1"/>
       <c r="B11" s="26"/>
-      <c r="C11" s="43"/>
-      <c r="D11" s="43"/>
+      <c r="C11" s="42"/>
+      <c r="D11" s="42"/>
       <c r="E11" s="26"/>
       <c r="F11" s="26"/>
       <c r="G11" s="26"/>
@@ -1078,8 +1100,8 @@
     <row r="12" spans="1:13" ht="30" customHeight="1">
       <c r="A12" s="1"/>
       <c r="B12" s="26"/>
-      <c r="C12" s="43"/>
-      <c r="D12" s="43"/>
+      <c r="C12" s="42"/>
+      <c r="D12" s="42"/>
       <c r="E12" s="26"/>
       <c r="F12" s="26"/>
       <c r="G12" s="26"/>
@@ -1092,8 +1114,8 @@
     <row r="13" spans="1:13" ht="30" customHeight="1">
       <c r="A13" s="1"/>
       <c r="B13" s="26"/>
-      <c r="C13" s="43"/>
-      <c r="D13" s="43"/>
+      <c r="C13" s="42"/>
+      <c r="D13" s="42"/>
       <c r="E13" s="26"/>
       <c r="F13" s="26"/>
       <c r="G13" s="26"/>
@@ -1106,8 +1128,8 @@
     <row r="14" spans="1:13" ht="30" customHeight="1">
       <c r="A14" s="1"/>
       <c r="B14" s="26"/>
-      <c r="C14" s="43"/>
-      <c r="D14" s="43"/>
+      <c r="C14" s="42"/>
+      <c r="D14" s="42"/>
       <c r="E14" s="26"/>
       <c r="F14" s="26"/>
       <c r="G14" s="26"/>
@@ -1119,8 +1141,8 @@
     </row>
     <row r="15" spans="1:13" s="1" customFormat="1" ht="30" customHeight="1">
       <c r="B15" s="26"/>
-      <c r="C15" s="43"/>
-      <c r="D15" s="43"/>
+      <c r="C15" s="42"/>
+      <c r="D15" s="42"/>
       <c r="E15" s="26"/>
       <c r="F15" s="26"/>
       <c r="G15" s="26"/>
@@ -1132,8 +1154,8 @@
     </row>
     <row r="16" spans="1:13" s="1" customFormat="1" ht="30" customHeight="1">
       <c r="B16" s="26"/>
-      <c r="C16" s="43"/>
-      <c r="D16" s="43"/>
+      <c r="C16" s="42"/>
+      <c r="D16" s="42"/>
       <c r="E16" s="26"/>
       <c r="F16" s="26"/>
       <c r="G16" s="26"/>
@@ -1146,8 +1168,8 @@
     <row r="17" spans="1:12" ht="30" customHeight="1">
       <c r="A17" s="1"/>
       <c r="B17" s="26"/>
-      <c r="C17" s="43"/>
-      <c r="D17" s="43"/>
+      <c r="C17" s="42"/>
+      <c r="D17" s="42"/>
       <c r="E17" s="26"/>
       <c r="F17" s="26"/>
       <c r="G17" s="26"/>
@@ -1159,8 +1181,8 @@
     </row>
     <row r="18" spans="1:12" s="1" customFormat="1" ht="30" customHeight="1">
       <c r="B18" s="26"/>
-      <c r="C18" s="43"/>
-      <c r="D18" s="43"/>
+      <c r="C18" s="42"/>
+      <c r="D18" s="42"/>
       <c r="E18" s="26"/>
       <c r="F18" s="26"/>
       <c r="G18" s="26"/>
@@ -1172,8 +1194,8 @@
     </row>
     <row r="19" spans="1:12" s="1" customFormat="1" ht="30" customHeight="1">
       <c r="B19" s="26"/>
-      <c r="C19" s="43"/>
-      <c r="D19" s="43"/>
+      <c r="C19" s="42"/>
+      <c r="D19" s="42"/>
       <c r="E19" s="26"/>
       <c r="F19" s="26"/>
       <c r="G19" s="26"/>
@@ -1185,8 +1207,8 @@
     </row>
     <row r="20" spans="1:12" s="1" customFormat="1" ht="30" customHeight="1">
       <c r="B20" s="26"/>
-      <c r="C20" s="43"/>
-      <c r="D20" s="43"/>
+      <c r="C20" s="42"/>
+      <c r="D20" s="42"/>
       <c r="E20" s="26"/>
       <c r="F20" s="26"/>
       <c r="G20" s="26"/>
@@ -1198,8 +1220,8 @@
     </row>
     <row r="21" spans="1:12" s="1" customFormat="1" ht="30" customHeight="1">
       <c r="B21" s="26"/>
-      <c r="C21" s="43"/>
-      <c r="D21" s="43"/>
+      <c r="C21" s="42"/>
+      <c r="D21" s="42"/>
       <c r="E21" s="26"/>
       <c r="F21" s="26"/>
       <c r="G21" s="26"/>
@@ -1210,118 +1232,118 @@
       <c r="L21" s="26"/>
     </row>
     <row r="22" spans="1:12" s="1" customFormat="1" ht="30" customHeight="1">
-      <c r="B22" s="47" t="s">
-        <v>25</v>
-      </c>
-      <c r="C22" s="48"/>
-      <c r="D22" s="48"/>
-      <c r="E22" s="48"/>
-      <c r="F22" s="40"/>
+      <c r="B22" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C22" s="29"/>
+      <c r="D22" s="29"/>
+      <c r="E22" s="29"/>
+      <c r="F22" s="30"/>
       <c r="G22" s="10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H22" s="5"/>
       <c r="I22" s="11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="J22" s="5"/>
       <c r="K22" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="L22" s="6"/>
+    </row>
+    <row r="23" spans="1:12" s="1" customFormat="1" ht="30" customHeight="1">
+      <c r="B23" s="31"/>
+      <c r="C23" s="32"/>
+      <c r="D23" s="32"/>
+      <c r="E23" s="32"/>
+      <c r="F23" s="33"/>
+      <c r="G23" s="7"/>
+      <c r="H23" s="53"/>
+      <c r="I23" s="54"/>
+      <c r="J23" s="54"/>
+      <c r="K23" s="54"/>
+      <c r="L23" s="55"/>
+    </row>
+    <row r="24" spans="1:12" s="1" customFormat="1" ht="12.7" customHeight="1">
+      <c r="B24" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="L22" s="6"/>
-    </row>
-    <row r="23" spans="1:12" s="1" customFormat="1" ht="30" customHeight="1">
-      <c r="B23" s="41"/>
-      <c r="C23" s="42"/>
-      <c r="D23" s="42"/>
-      <c r="E23" s="42"/>
-      <c r="F23" s="31"/>
-      <c r="G23" s="7"/>
-      <c r="H23" s="35"/>
-      <c r="I23" s="36"/>
-      <c r="J23" s="36"/>
-      <c r="K23" s="36"/>
-      <c r="L23" s="37"/>
-    </row>
-    <row r="24" spans="1:12" s="1" customFormat="1" ht="12.7" customHeight="1">
-      <c r="B24" s="49" t="s">
-        <v>23</v>
-      </c>
-      <c r="C24" s="36"/>
-      <c r="D24" s="36"/>
-      <c r="E24" s="36"/>
-      <c r="F24" s="36"/>
-      <c r="G24" s="37"/>
-      <c r="H24" s="38"/>
-      <c r="I24" s="39"/>
-      <c r="J24" s="39"/>
-      <c r="K24" s="39"/>
-      <c r="L24" s="40"/>
+      <c r="C24" s="35"/>
+      <c r="D24" s="35"/>
+      <c r="E24" s="35"/>
+      <c r="F24" s="35"/>
+      <c r="G24" s="36"/>
+      <c r="H24" s="56"/>
+      <c r="I24" s="57"/>
+      <c r="J24" s="57"/>
+      <c r="K24" s="57"/>
+      <c r="L24" s="58"/>
     </row>
     <row r="25" spans="1:12" s="1" customFormat="1" ht="12.7" customHeight="1">
-      <c r="B25" s="38"/>
-      <c r="C25" s="39"/>
-      <c r="D25" s="39"/>
-      <c r="E25" s="39"/>
-      <c r="F25" s="39"/>
-      <c r="G25" s="40"/>
-      <c r="H25" s="38"/>
-      <c r="I25" s="39"/>
-      <c r="J25" s="39"/>
-      <c r="K25" s="39"/>
-      <c r="L25" s="40"/>
+      <c r="B25" s="37"/>
+      <c r="C25" s="38"/>
+      <c r="D25" s="38"/>
+      <c r="E25" s="38"/>
+      <c r="F25" s="38"/>
+      <c r="G25" s="30"/>
+      <c r="H25" s="56"/>
+      <c r="I25" s="57"/>
+      <c r="J25" s="57"/>
+      <c r="K25" s="57"/>
+      <c r="L25" s="58"/>
     </row>
     <row r="26" spans="1:12" s="1" customFormat="1" ht="12.7" customHeight="1">
-      <c r="B26" s="38"/>
-      <c r="C26" s="39"/>
-      <c r="D26" s="39"/>
-      <c r="E26" s="39"/>
-      <c r="F26" s="39"/>
-      <c r="G26" s="40"/>
-      <c r="H26" s="38"/>
-      <c r="I26" s="39"/>
-      <c r="J26" s="39"/>
-      <c r="K26" s="39"/>
-      <c r="L26" s="40"/>
+      <c r="B26" s="37"/>
+      <c r="C26" s="38"/>
+      <c r="D26" s="38"/>
+      <c r="E26" s="38"/>
+      <c r="F26" s="38"/>
+      <c r="G26" s="30"/>
+      <c r="H26" s="56"/>
+      <c r="I26" s="57"/>
+      <c r="J26" s="57"/>
+      <c r="K26" s="57"/>
+      <c r="L26" s="58"/>
     </row>
     <row r="27" spans="1:12" s="1" customFormat="1" ht="12.7" customHeight="1">
-      <c r="B27" s="38"/>
-      <c r="C27" s="39"/>
-      <c r="D27" s="39"/>
-      <c r="E27" s="39"/>
-      <c r="F27" s="39"/>
-      <c r="G27" s="40"/>
-      <c r="H27" s="38"/>
-      <c r="I27" s="39"/>
-      <c r="J27" s="39"/>
-      <c r="K27" s="39"/>
-      <c r="L27" s="40"/>
+      <c r="B27" s="37"/>
+      <c r="C27" s="38"/>
+      <c r="D27" s="38"/>
+      <c r="E27" s="38"/>
+      <c r="F27" s="38"/>
+      <c r="G27" s="30"/>
+      <c r="H27" s="56"/>
+      <c r="I27" s="57"/>
+      <c r="J27" s="57"/>
+      <c r="K27" s="57"/>
+      <c r="L27" s="58"/>
     </row>
     <row r="28" spans="1:12" s="1" customFormat="1" ht="12.7" customHeight="1">
-      <c r="B28" s="38"/>
-      <c r="C28" s="39"/>
-      <c r="D28" s="39"/>
-      <c r="E28" s="39"/>
-      <c r="F28" s="39"/>
-      <c r="G28" s="40"/>
-      <c r="H28" s="38"/>
-      <c r="I28" s="39"/>
-      <c r="J28" s="39"/>
-      <c r="K28" s="39"/>
-      <c r="L28" s="40"/>
+      <c r="B28" s="37"/>
+      <c r="C28" s="38"/>
+      <c r="D28" s="38"/>
+      <c r="E28" s="38"/>
+      <c r="F28" s="38"/>
+      <c r="G28" s="30"/>
+      <c r="H28" s="56"/>
+      <c r="I28" s="57"/>
+      <c r="J28" s="57"/>
+      <c r="K28" s="57"/>
+      <c r="L28" s="58"/>
     </row>
     <row r="29" spans="1:12" s="1" customFormat="1" ht="12.7" customHeight="1">
-      <c r="B29" s="41"/>
-      <c r="C29" s="42"/>
-      <c r="D29" s="42"/>
-      <c r="E29" s="42"/>
-      <c r="F29" s="42"/>
-      <c r="G29" s="31"/>
-      <c r="H29" s="41"/>
-      <c r="I29" s="42"/>
-      <c r="J29" s="42"/>
-      <c r="K29" s="42"/>
-      <c r="L29" s="31"/>
+      <c r="B29" s="31"/>
+      <c r="C29" s="32"/>
+      <c r="D29" s="32"/>
+      <c r="E29" s="32"/>
+      <c r="F29" s="32"/>
+      <c r="G29" s="33"/>
+      <c r="H29" s="59"/>
+      <c r="I29" s="60"/>
+      <c r="J29" s="60"/>
+      <c r="K29" s="60"/>
+      <c r="L29" s="61"/>
     </row>
     <row r="30" spans="1:12" s="1" customFormat="1" ht="12.7" customHeight="1">
       <c r="B30" s="8"/>
@@ -1357,18 +1379,6 @@
     <row r="38"/>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="B22:F23"/>
-    <mergeCell ref="B24:G29"/>
-    <mergeCell ref="B1:D2"/>
-    <mergeCell ref="F1:J2"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="F5:K5"/>
     <mergeCell ref="M4:M5"/>
     <mergeCell ref="L4:L5"/>
     <mergeCell ref="C6:D6"/>
@@ -1385,6 +1395,18 @@
     <mergeCell ref="C15:D15"/>
     <mergeCell ref="C4:G4"/>
     <mergeCell ref="C3:E3"/>
+    <mergeCell ref="B22:F23"/>
+    <mergeCell ref="B24:G29"/>
+    <mergeCell ref="B1:D2"/>
+    <mergeCell ref="F1:J2"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="F5:K5"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <printOptions horizontalCentered="1"/>

</xml_diff>